<commit_message>
Cập nhật K76.A11 - 14:40 28/4/26
</commit_message>
<xml_diff>
--- a/data/danhsach.xlsx
+++ b/data/danhsach.xlsx
@@ -457,10 +457,10 @@
         <v>Lê Thế Anh</v>
       </c>
       <c r="C2">
-        <v>10.734025</v>
+        <v>10.733988</v>
       </c>
       <c r="D2">
-        <v>106.640794</v>
+        <v>106.640812</v>
       </c>
       <c r="E2" t="str">
         <v/>

</xml_diff>